<commit_message>
docs(user-stories): fix inconsistencies in HU-01, HU-11, HU-13, HU-16 and HU-32
</commit_message>
<xml_diff>
--- a/docs/FastRoute_Historias.xlsx
+++ b/docs/FastRoute_Historias.xlsx
@@ -608,7 +608,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Como administrador,quiero registrar en el sistema de FastRouteCO las empresas contratistas para que estas mejoren la eficiencia de envíos o reclamos.</t>
+          <t>Como administrador,quiero registrar en el sistema de FastRouteCO las empresas contratistas para que estas mejoren la eficiencia de sus entregas y recogidas.</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -1054,7 +1054,7 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Como supervisor de la empresa contratista, quiero poder tener una comunicación directa con los conductores de las rutas, para poder solucionar cualquier inconveniente con el sistema FastRouteCO o duda que tenga dicho conductor</t>
+          <t>Como supervisor de la empresa contratista, quiero poder tener una comunicación directa con los conductores de las rutas, para poder resolver las incidencias o dudas que tenga dicho conductor durante la ruta</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
@@ -1145,7 +1145,7 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>CA01: El conductor debe poder visualizar sus rutas asignadas, un apartado de reclamos o comunicacion con el sistema o el supervisor de la ruta.
+          <t>CA01: El conductor debe poder visualizar sus rutas asignadas, un apartado para reportar incidencias o dudas y comunicarse con el supervisor de la ruta.
 CA02:Apartado que permita notificar el comienzo de una ruta</t>
         </is>
       </c>
@@ -1154,7 +1154,7 @@
           <t>R01:Tener acceso al sistema
 R02: Se requiere conexión para sincronizar datos y para el seguimiento en tiempo real. Sin conexión aplica lo definido en la HU-36
 R03: Sea conductor
-R04: La empresa tenga contrato</t>
+R04: La empresa debe estar activa. Para iniciar una ruta aplica además lo definido en la HU-30 (R03)</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
@@ -1295,7 +1295,7 @@
         <is>
           <t>R01:Solo el administrador de la empresa puede gestionar el plan de suscripción
 R02: No se pueden usar solicitudes si el saldo es cero y no se han adquirido adicionales
-R03: Las solicitudes del plan aplican solo a la modalidad de suscripción; en pago por uso cada optimización se cobra (HU-37)</t>
+R03: Las solicitudes aplican a los planes de suscripción y al Free Trial; en pago por uso cada optimización se cobra (HU-37)</t>
         </is>
       </c>
       <c r="H18" s="3" t="inlineStr">
@@ -2017,7 +2017,7 @@
       </c>
       <c r="G34" s="3" t="inlineStr">
         <is>
-          <t>R01: La empresa debe tener el módulo escolar (incluido en Premium, adquirido en Pro o de prueba en el Free Trial)
+          <t>R01: La empresa debe tener el módulo escolar (incluido en Premium, adquirido en Pro o en pago por uso, o de prueba en el Free Trial)
 R02: Solo el supervisor logístico o el cliente empresa pueden gestionar estudiantes</t>
         </is>
       </c>

</xml_diff>